<commit_message>
Slim the CUH final-ask workbook after Josh's second inventory reply
The Discharge dashboard covers ward discharges by hour/day-of-week, and
occupancy comes from published KH03 (the consistent denominator CUH said
they lack) - so both leave the human ask. What remains from a person at
CUH: Capacity counts + four quick questions; the Areas grid becomes an
optional confirm (pre-filled from CHEQS extracts on arrival). Same
filename so only one version circulates.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWC8yvMKU2mXFbMKfvB2cP
</commit_message>
<xml_diff>
--- a/docs/cuh_minimum_data.xlsx
+++ b/docs/cuh_minimum_data.xlsx
@@ -9,9 +9,9 @@
   <sheets>
     <sheet name="READ ME" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Overview" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Areas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Capacity" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Downstream" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Capacity" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Questions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Areas" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +426,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>CAMBRIDGE ED (CUH / RGT) - MINIMUM DATA COLLECTION</t>
+          <t>CAMBRIDGE ED (CUH / RGT) - FINAL ASK  (v2, supersedes any earlier copy)</t>
         </is>
       </c>
     </row>
@@ -436,76 +436,80 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Purpose: everything on this file is data ONLY CUH can tell us. It is the</t>
+          <t>Everything else is already agreed elsewhere:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>complete ask for the first deliverable - the ED flow view with headline</t>
+          <t xml:space="preserve">  - CHEQS extracts + Discharge dashboard: with Josh (arrivals, area flows,</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>metrics (control tower). Fillable in one 30-45 min chat with the ED ops manager.</t>
+          <t xml:space="preserve">    patient moves, timings, imaging counts, MH, monthly performance,</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    discharges by hour).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Everything else - attendances, beds, occupancy, 4-hour performance, arrival</t>
+          <t xml:space="preserve">  - Published NHS data: attendances, 4-hour/12-hour performance, and</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>patterns, acuity mix - comes from published NHS data. No workforce data,</t>
+          <t xml:space="preserve">    G&amp;A beds + occupancy (KH03 return - no occupancy work needed at CUH).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>no patient-level data, no identifiers.</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>This file is ONLY what no dashboard or publication can tell us:</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3 tabs to fill:</t>
+          <t xml:space="preserve">  Capacity   - REQUIRED: physical counts of each space.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Areas      - yes/no for every row + opening hours</t>
+          <t xml:space="preserve">  Questions  - REQUIRED: four quick answers (rough figures are fine).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capacity   - physical counts (how many of each space)</t>
+          <t xml:space="preserve">  Areas      - OPTIONAL: we pre-fill this from the CHEQS extracts and ask</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Downstream - 4 quick questions (rough figures are fine)</t>
+          <t xml:space="preserve">               you only to confirm; fill it now only if quicker.</t>
         </is>
       </c>
     </row>
@@ -515,14 +519,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Anything left blank stays a clearly-labelled model assumption - never a</t>
+          <t>Blank = unknown is fine; it stays a clearly-labelled model assumption.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>silent guess. Please don't estimate: blank is better than approximate.</t>
+          <t>Please don't estimate physical counts - blank beats approximate.</t>
         </is>
       </c>
     </row>
@@ -583,7 +587,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t># Do not edit this tab - published NHS data fills the rest.</t>
+          <t># Do not edit - published NHS data fills everything numeric.</t>
         </is>
       </c>
     </row>
@@ -593,6 +597,307 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resource_key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>your_count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>belongs to</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>utc_room</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Co-located Urgent Treatment Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>minor_injury_space</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Core ED (always present)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fit_to_sit_chair</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ambulatory ‘fit to sit’ area</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cubicle</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Core ED (always present)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>resus_bay</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Core ED (always present)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paeds_cubicle</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Children’s area / PAU</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ct_scanner</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Core ED (always present)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>xray_room</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Core ED (always present)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>eemac_space</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EEMAC (extended emergency ambulatory care)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sdec_chair</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Specialty Same-Day Emergency Care (SDEC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>cdu_bed</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Clinical Decision Unit (CDU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>fau_bed</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Frailty unit (FAU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>mh_assessment_room</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mental-health liaison / MHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>handover_bay</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Core ED (always present)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t># REQUIRED. How many physically exist (not how many are staffed open).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t># Skip rows for areas the ED does not have. Blank = unknown.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>question</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1. Does CHEQS (and everything in this file) cover the ADULT Type 1 ED only, with the paediatric ED separate? (yes/no)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2. Roughly how many patients per day can community / virtual-ward services take from the hospital? (number)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3. Are there any ED areas that exist but would NOT show up as locations in CHEQS? (list, or 'none')</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4. Any areas whose opening hours differ from when arrivals appear in CHEQS - e.g. stops accepting at 18:00 but open later? (list, or 'none')</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t># REQUIRED - four answers, rough is fine.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -773,315 +1078,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve"># Answer yes/no for EVERY row. Hours: 24/7 = 0 and 24; blank hours = </t>
+          <t># OPTIONAL - we pre-fill this from the CHEQS extracts and only ask you to</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t># sensible defaults (rat 0-24, utc 8-24, fit_to_sit 8-22, paeds 8-22, eemac 8-22, sdec 8-20, cdu 0-24, frailty 8-18, mh 0-24)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>resource_key</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>your_count</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>belongs to</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>utc_room</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Co-located Urgent Treatment Centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>minor_injury_space</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Core ED (always present)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>fit_to_sit_chair</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Ambulatory ‘fit to sit’ area</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>cubicle</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Core ED (always present)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>resus_bay</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Core ED (always present)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paeds_cubicle</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Children’s area / PAU</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ct_scanner</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Core ED (always present)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>xray_room</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Core ED (always present)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>eemac_space</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>EEMAC (extended emergency ambulatory care)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>sdec_chair</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Specialty Same-Day Emergency Care (SDEC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>cdu_bed</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Clinical Decision Unit (CDU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>fau_bed</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Frailty unit (FAU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>mh_assessment_room</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Mental-health liaison / MHED</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>handover_bay</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Core ED (always present)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t># How many physically exist (not how many are staffed/open).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t># Skip rows for areas answered 'no' on the Areas tab. Blank = unknown.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="95" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Roughly how many patients are discharged from the inpatient wards on a typical day?</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Roughly what share of those discharges happen before 1pm? (%)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>How many patients per day can community / virtual-ward services take?</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Does everything in this file cover the ADULT Type 1 ED only (paediatric ED separate)? (yes/no)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t># These make the 'waiting for a bed' part of the flow real. Rough figures are fine.</t>
+          <t># confirm the mapping. Fill now only if that is quicker for you.</t>
         </is>
       </c>
     </row>

</xml_diff>